<commit_message>
time and text based version of main
zamanlama ve metin benzerliğine göre karakter atamalarını yapmayı hedefledi fakat karakter atamaları olmadı ve çalışma süresi fazla uzun
</commit_message>
<xml_diff>
--- a/text2_log.xlsx
+++ b/text2_log.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C43"/>
+  <dimension ref="A1:D43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,6 +444,11 @@
           <t>Turkish</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>character</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -461,6 +466,11 @@
           <t xml:space="preserve"> Büyümlesin  efendim,  beni  şartmışsınız.  Ha,  lala.  Çalışanlara  tembih  et  lütfen.  Hiçbir  şey  israf  etmesinler.  Zor  günlerden  geçeceğiz.  Babı  efendim.</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -478,6 +488,11 @@
           <t xml:space="preserve"> Eee  bir  de  şey  soracaktım.  Bugün  bolstacı  geldi  mi?  Gel  de  efendim.</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -495,6 +510,11 @@
           <t xml:space="preserve"> Bir  tattan  haber  var.  Yok.  Ama  merak  etmeyin.  Yarın  öbür  gün.  Gelir.</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -512,6 +532,11 @@
           <t xml:space="preserve"> Sağ  ol.</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -529,6 +554,11 @@
           <t xml:space="preserve"> Sağ  ol.  Biliyor  musun  Aşı?  Annem  beni  evlendirdiğinde  o  beş  yaşındaydım.</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -546,6 +576,11 @@
           <t xml:space="preserve"> O  yılda  hamile  kaldım.  Ha.</t>
         </is>
       </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -563,6 +598,11 @@
           <t xml:space="preserve"> Daha  kendim  çocukluğum  yani.</t>
         </is>
       </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -580,6 +620,11 @@
           <t xml:space="preserve"> Hamileliğim  ramağına  denk  gelmiştim.</t>
         </is>
       </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -597,6 +642,11 @@
           <t xml:space="preserve"> Bir  gece  sabır  da.  Davucunun  sesini  duyunca  sokağı  fırladım.  Ben  de  göbeğimi  uğra  uğra  dolaştım.</t>
         </is>
       </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -614,6 +664,11 @@
           <t xml:space="preserve"> Reşar  da  oynamak  isterdim.</t>
         </is>
       </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -631,6 +686,11 @@
           <t xml:space="preserve"> İzin  mermezlerdi.</t>
         </is>
       </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -648,6 +708,11 @@
           <t xml:space="preserve"> Artık  evlesin  çocuk  değilsin  derlerdi.  Sen  çocuk  değilsin  değilce.  Çocukluk  bitiyormuş  ki.</t>
         </is>
       </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -665,6 +730,11 @@
           <t xml:space="preserve"> Ama  bir  tatdayın.  Ah  benim  bir  tamağa.</t>
         </is>
       </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -682,6 +752,11 @@
           <t xml:space="preserve"> Ama  bana  hiç  kıyamazdı.</t>
         </is>
       </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -699,6 +774,11 @@
           <t xml:space="preserve"> Bütün  çocuklar  sokakta  oynarken.  Bu  benimle  evde  oturup.</t>
         </is>
       </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -716,6 +796,11 @@
           <t xml:space="preserve"> Gizli  gizli  oyun  kul  artık.  Ah  bir  tatım  benim.</t>
         </is>
       </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -733,6 +818,11 @@
           <t xml:space="preserve"> Hiç  kıyamazdı  bana  hiç.</t>
         </is>
       </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -750,6 +840,11 @@
           <t xml:space="preserve"> Bazen  de  hatırımı  kırmamak  için.  Bebekler  bunlar.</t>
         </is>
       </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -767,6 +862,11 @@
           <t xml:space="preserve"> Merak  etmeyin.  Bir  tatdayım  sağ  salim  dönecektir.</t>
         </is>
       </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -784,6 +884,11 @@
           <t xml:space="preserve"> Hem  onun  olduğu  taraflarda  hareket  yok  ki.</t>
         </is>
       </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -801,6 +906,11 @@
           <t xml:space="preserve"> İnşallah.</t>
         </is>
       </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -818,6 +928,11 @@
           <t xml:space="preserve"> Komitacının  nerede  olduğu  belli  olmuyor  ya.</t>
         </is>
       </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -835,6 +950,11 @@
           <t xml:space="preserve"> Anneciğim  sahil  poşalar  haber  verdiniz  mi?  Ne  haberi?  Ev  ziyaretini  sırası  değil  tehir  edelim  demiştiniz  yani.</t>
         </is>
       </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -852,6 +972,11 @@
           <t xml:space="preserve"> Tamam  tamam.  Ben  öyle  düşünüyordum  ama  bana  öyle  düşünmüyor.  Büyük  bir  ayaklama  değil  o  dedi.  Gidilecek  yani.  Evet.  Peki  o  zaman  ben  annesi  engema  haber  vereyim.  İptal  oldu  zannediyor  çünkü.  Söyle  ona.  Ne  değilsin  de  hazırlasın.</t>
         </is>
       </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -869,6 +994,11 @@
           <t xml:space="preserve"> Anneciğim  kalkalım  mı?  Geç  kalıyoruz  kalkalım.</t>
         </is>
       </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -886,6 +1016,11 @@
           <t xml:space="preserve"> Evet.</t>
         </is>
       </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -903,6 +1038,11 @@
           <t xml:space="preserve"> Evet.  Tamam  var  ya.  Geçim  emin  iyilişte  bir  yolcu  edeceğiz.  Gelecek  misınız?</t>
         </is>
       </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -920,6 +1060,11 @@
           <t xml:space="preserve"> Yok  gelmeyeceğim.  Mutar  ağa  uysuz.  Hala  uyumadı.  Uyumadı  mı?  Hay  Allah.</t>
         </is>
       </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -937,6 +1082,11 @@
           <t xml:space="preserve"> Sen  söylersin  onlara.  Ben  emin  beliye  yollacaklar  deliyorum.  Peki  söylerim.</t>
         </is>
       </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -954,6 +1104,11 @@
           <t xml:space="preserve"> Ee  bir  de...  Annem  dedi  ki...  Sahir  Paşalara  giderken  annesi  hediyesini  hazırlesin.</t>
         </is>
       </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -971,6 +1126,11 @@
           <t xml:space="preserve"> Böylim  gündür  çıksın.</t>
         </is>
       </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -988,6 +1148,11 @@
           <t xml:space="preserve"> Tek  bir  kelime  etmeden.</t>
         </is>
       </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1005,6 +1170,11 @@
           <t xml:space="preserve"> Babana  tekrar  söyledim.  Al  böyleyken  evin  masraflarına  katkıda  bulunmazsam  rahat  edemem  diye.</t>
         </is>
       </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1022,6 +1192,11 @@
           <t xml:space="preserve"> Ama  yine  reddetti.</t>
         </is>
       </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1039,6 +1214,11 @@
           <t xml:space="preserve"> Sen  bunu  annene  ver,  ben  gidince.</t>
         </is>
       </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1056,6 +1236,11 @@
           <t xml:space="preserve"> Babana  söylemesin.</t>
         </is>
       </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1073,6 +1258,11 @@
           <t xml:space="preserve"> Her  ay  göndereceğim  bir  bu  kadar.</t>
         </is>
       </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1090,6 +1280,11 @@
           <t xml:space="preserve"> Siz  aşağın.  Ram  Paşa  evi  leide  gidiyor.</t>
         </is>
       </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1107,6 +1302,11 @@
           <t xml:space="preserve"> Siz  aşağın.</t>
         </is>
       </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1124,6 +1324,11 @@
           <t xml:space="preserve"> Siz  aşağın.</t>
         </is>
       </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1141,6 +1346,11 @@
           <t xml:space="preserve"> Ben  sizi  görmek  istediğimi  konuşmak  istiyorum  size.  Dün  müsait  değilim  şu  an.</t>
         </is>
       </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1156,6 +1366,11 @@
       <c r="C43" t="inlineStr">
         <is>
           <t xml:space="preserve"> Çok  mühimse  söylesin  canım.</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Unknown</t>
         </is>
       </c>
     </row>

</xml_diff>